<commit_message>
reference bug in spreadsheets fixed
</commit_message>
<xml_diff>
--- a/AvantisChannelList.xlsx
+++ b/AvantisChannelList.xlsx
@@ -14,9 +14,6 @@
     <sheet name="Mixer Config" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Misc" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -49,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5909" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6245" uniqueCount="424">
   <si>
     <t xml:space="preserve">Enabled</t>
   </si>
@@ -1863,148 +1860,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Channels"/>
-      <sheetName val="Sockets"/>
-      <sheetName val="Groups"/>
-      <sheetName val="Mixer Config"/>
-      <sheetName val="Misc"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2">
-        <row r="2">
-          <cell r="P2" t="str">
-            <v>Grp1</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="U2" t="str">
-            <v>StGrp1</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="P3" t="str">
-            <v>Grp2</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="U3" t="str">
-            <v>StGrp2</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="P4" t="str">
-            <v>Grp3</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="U4" t="str">
-            <v>StGrp3</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="P5" t="str">
-            <v>Grp4</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="U5" t="str">
-            <v>StGrp4</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="P6" t="str">
-            <v>Grp5</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="U6" t="str">
-            <v>StGrp5</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="P7" t="str">
-            <v>Grp6</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="U7" t="str">
-            <v>StGrp6</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="P8" t="str">
-            <v>Grp7</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="U8" t="str">
-            <v>StGrp7</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="P9" t="str">
-            <v>Grp8</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="U9" t="str">
-            <v>StGrp8</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="P10" t="str">
-            <v>Grp9</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="U10" t="str">
-            <v>StGrp9</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="P11" t="str">
-            <v>Grp10</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="U11" t="str">
-            <v>StGrp10</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="P12" t="str">
-            <v>Grp11</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="U12" t="str">
-            <v>StGrp11</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="P13" t="str">
-            <v>Grp12</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="U13" t="str">
-            <v>StGrp12</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
   <a:themeElements>
@@ -2189,100 +2044,100 @@
       </c>
       <c r="O1" s="5"/>
       <c r="P1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp1 - ",[1]Groups!P2)</f>
+        <f aca="false">CONCATENATE("Grp1 - ",Groups!P2)</f>
         <v>Grp1 - Grp1</v>
       </c>
       <c r="Q1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp2 - ",[1]Groups!P3)</f>
+        <f aca="false">CONCATENATE("Grp2 - ",Groups!P3)</f>
         <v>Grp2 - Grp2</v>
       </c>
       <c r="R1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp3 - ",[1]Groups!P4)</f>
+        <f aca="false">CONCATENATE("Grp3 - ",Groups!P4)</f>
         <v>Grp3 - Grp3</v>
       </c>
       <c r="S1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp4 - ",[1]Groups!P5)</f>
+        <f aca="false">CONCATENATE("Grp4 - ",Groups!P5)</f>
         <v>Grp4 - Grp4</v>
       </c>
       <c r="T1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp5 - ",[1]Groups!P6)</f>
+        <f aca="false">CONCATENATE("Grp5 - ",Groups!P6)</f>
         <v>Grp5 - Grp5</v>
       </c>
       <c r="U1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp6 - ",[1]Groups!P7)</f>
+        <f aca="false">CONCATENATE("Grp6 - ",Groups!P7)</f>
         <v>Grp6 - Grp6</v>
       </c>
       <c r="V1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp7 - ",[1]Groups!P8)</f>
+        <f aca="false">CONCATENATE("Grp7 - ",Groups!P8)</f>
         <v>Grp7 - Grp7</v>
       </c>
       <c r="W1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp8 - ",[1]Groups!$P9)</f>
+        <f aca="false">CONCATENATE("Grp8 - ",Groups!P9)</f>
         <v>Grp8 - Grp8</v>
       </c>
       <c r="X1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp9 - ",[1]Groups!$P10)</f>
+        <f aca="false">CONCATENATE("Grp9 - ",Groups!P10)</f>
         <v>Grp9 - Grp9</v>
       </c>
       <c r="Y1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp10 - ",[1]Groups!$P11)</f>
+        <f aca="false">CONCATENATE("Grp10 - ",Groups!P11)</f>
         <v>Grp10 - Grp10</v>
       </c>
       <c r="Z1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp11 - ",[1]Groups!$P12)</f>
+        <f aca="false">CONCATENATE("Grp11 - ",Groups!P12)</f>
         <v>Grp11 - Grp11</v>
       </c>
       <c r="AA1" s="8" t="str">
-        <f aca="false">CONCATENATE("Grp12 - ",[1]Groups!$P13)</f>
+        <f aca="false">CONCATENATE("Grp12 - ",Groups!P13)</f>
         <v>Grp12 - Grp12</v>
       </c>
       <c r="AB1" s="5"/>
       <c r="AC1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp1 - ",[1]Groups!U2)</f>
+        <f aca="false">CONCATENATE("StGrp1 - ",Groups!U2)</f>
         <v>StGrp1 - StGrp1</v>
       </c>
       <c r="AD1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp2 - ",[1]Groups!U3)</f>
+        <f aca="false">CONCATENATE("StGrp2 - ",Groups!U3)</f>
         <v>StGrp2 - StGrp2</v>
       </c>
       <c r="AE1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp3 - ",[1]Groups!U4)</f>
+        <f aca="false">CONCATENATE("StGrp3 - ",Groups!U4)</f>
         <v>StGrp3 - StGrp3</v>
       </c>
       <c r="AF1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp4 - ",[1]Groups!U5)</f>
+        <f aca="false">CONCATENATE("StGrp4 - ",Groups!U5)</f>
         <v>StGrp4 - StGrp4</v>
       </c>
       <c r="AG1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp5 - ",[1]Groups!U6)</f>
+        <f aca="false">CONCATENATE("StGrp5 - ",Groups!U6)</f>
         <v>StGrp5 - StGrp5</v>
       </c>
       <c r="AH1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp6 - ",[1]Groups!U7)</f>
+        <f aca="false">CONCATENATE("StGrp6 - ",Groups!U7)</f>
         <v>StGrp6 - StGrp6</v>
       </c>
       <c r="AI1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp7 - ",[1]Groups!U8)</f>
+        <f aca="false">CONCATENATE("StGrp7 - ",Groups!U8)</f>
         <v>StGrp7 - StGrp7</v>
       </c>
       <c r="AJ1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp8 - ",[1]Groups!U9)</f>
+        <f aca="false">CONCATENATE("StGrp8 - ",Groups!U9)</f>
         <v>StGrp8 - StGrp8</v>
       </c>
       <c r="AK1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp9 - ",[1]Groups!U10)</f>
+        <f aca="false">CONCATENATE("StGrp9 - ",Groups!U10)</f>
         <v>StGrp9 - StGrp9</v>
       </c>
       <c r="AL1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp10 - ",[1]Groups!U11)</f>
+        <f aca="false">CONCATENATE("StGrp10 - ",Groups!U11)</f>
         <v>StGrp10 - StGrp10</v>
       </c>
       <c r="AM1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp11 - ",[1]Groups!U12)</f>
+        <f aca="false">CONCATENATE("StGrp11 - ",Groups!U12)</f>
         <v>StGrp11 - StGrp11</v>
       </c>
       <c r="AN1" s="8" t="str">
-        <f aca="false">CONCATENATE("StGrp12 - ",[1]Groups!U13)</f>
+        <f aca="false">CONCATENATE("StGrp12 - ",Groups!U13)</f>
         <v>StGrp12 - StGrp12</v>
       </c>
       <c r="AO1" s="5"/>
@@ -2721,15 +2576,29 @@
       <c r="BO2" s="10"/>
       <c r="BP2" s="10"/>
       <c r="BR2" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS2" s="10"/>
-      <c r="BT2" s="10"/>
-      <c r="BU2" s="10"/>
-      <c r="BV2" s="10"/>
-      <c r="BW2" s="10"/>
-      <c r="BX2" s="10"/>
-      <c r="BY2" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX2" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY2" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA2" s="2" t="str">
         <f aca="false">IF(AS2="x","x",IF(AS2="-","-",""))</f>
         <v>x</v>
@@ -3083,15 +2952,29 @@
       <c r="BO3" s="10"/>
       <c r="BP3" s="10"/>
       <c r="BR3" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS3" s="10"/>
-      <c r="BT3" s="10"/>
-      <c r="BU3" s="10"/>
-      <c r="BV3" s="10"/>
-      <c r="BW3" s="10"/>
-      <c r="BX3" s="10"/>
-      <c r="BY3" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX3" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY3" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA3" s="2" t="str">
         <f aca="false">IF(AS3="x","x",IF(AS3="-","-",""))</f>
         <v>x</v>
@@ -3445,15 +3328,29 @@
       <c r="BO4" s="10"/>
       <c r="BP4" s="10"/>
       <c r="BR4" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS4" s="10"/>
-      <c r="BT4" s="10"/>
-      <c r="BU4" s="10"/>
-      <c r="BV4" s="10"/>
-      <c r="BW4" s="10"/>
-      <c r="BX4" s="10"/>
-      <c r="BY4" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX4" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY4" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA4" s="2" t="str">
         <f aca="false">IF(AS4="x","x",IF(AS4="-","-",""))</f>
         <v>x</v>
@@ -3807,15 +3704,29 @@
       <c r="BO5" s="10"/>
       <c r="BP5" s="10"/>
       <c r="BR5" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS5" s="10"/>
-      <c r="BT5" s="10"/>
-      <c r="BU5" s="10"/>
-      <c r="BV5" s="10"/>
-      <c r="BW5" s="10"/>
-      <c r="BX5" s="10"/>
-      <c r="BY5" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX5" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY5" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA5" s="2" t="str">
         <f aca="false">IF(AS5="x","x",IF(AS5="-","-",""))</f>
         <v>x</v>
@@ -4169,15 +4080,29 @@
       <c r="BO6" s="10"/>
       <c r="BP6" s="10"/>
       <c r="BR6" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS6" s="10"/>
-      <c r="BT6" s="10"/>
-      <c r="BU6" s="10"/>
-      <c r="BV6" s="10"/>
-      <c r="BW6" s="10"/>
-      <c r="BX6" s="10"/>
-      <c r="BY6" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX6" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY6" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA6" s="2" t="str">
         <f aca="false">IF(AS6="x","x",IF(AS6="-","-",""))</f>
         <v>x</v>
@@ -4531,15 +4456,29 @@
       <c r="BO7" s="10"/>
       <c r="BP7" s="10"/>
       <c r="BR7" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS7" s="10"/>
-      <c r="BT7" s="10"/>
-      <c r="BU7" s="10"/>
-      <c r="BV7" s="10"/>
-      <c r="BW7" s="10"/>
-      <c r="BX7" s="10"/>
-      <c r="BY7" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX7" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY7" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA7" s="2" t="str">
         <f aca="false">IF(AS7="x","x",IF(AS7="-","-",""))</f>
         <v>x</v>
@@ -4893,15 +4832,29 @@
       <c r="BO8" s="10"/>
       <c r="BP8" s="10"/>
       <c r="BR8" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS8" s="10"/>
-      <c r="BT8" s="10"/>
-      <c r="BU8" s="10"/>
-      <c r="BV8" s="10"/>
-      <c r="BW8" s="10"/>
-      <c r="BX8" s="10"/>
-      <c r="BY8" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX8" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY8" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA8" s="2" t="str">
         <f aca="false">IF(AS8="x","x",IF(AS8="-","-",""))</f>
         <v>x</v>
@@ -5255,15 +5208,29 @@
       <c r="BO9" s="10"/>
       <c r="BP9" s="10"/>
       <c r="BR9" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS9" s="10"/>
-      <c r="BT9" s="10"/>
-      <c r="BU9" s="10"/>
-      <c r="BV9" s="10"/>
-      <c r="BW9" s="10"/>
-      <c r="BX9" s="10"/>
-      <c r="BY9" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX9" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY9" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA9" s="2" t="str">
         <f aca="false">IF(AS9="x","x",IF(AS9="-","-",""))</f>
         <v>x</v>
@@ -5617,15 +5584,29 @@
       <c r="BO10" s="10"/>
       <c r="BP10" s="10"/>
       <c r="BR10" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS10" s="10"/>
-      <c r="BT10" s="10"/>
-      <c r="BU10" s="10"/>
-      <c r="BV10" s="10"/>
-      <c r="BW10" s="10"/>
-      <c r="BX10" s="10"/>
-      <c r="BY10" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX10" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY10" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA10" s="2" t="str">
         <f aca="false">IF(AS10="x","x",IF(AS10="-","-",""))</f>
         <v>x</v>
@@ -5979,15 +5960,29 @@
       <c r="BO11" s="10"/>
       <c r="BP11" s="10"/>
       <c r="BR11" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS11" s="10"/>
-      <c r="BT11" s="10"/>
-      <c r="BU11" s="10"/>
-      <c r="BV11" s="10"/>
-      <c r="BW11" s="10"/>
-      <c r="BX11" s="10"/>
-      <c r="BY11" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX11" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY11" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA11" s="2" t="str">
         <f aca="false">IF(AS11="x","x",IF(AS11="-","-",""))</f>
         <v>x</v>
@@ -6341,15 +6336,29 @@
       <c r="BO12" s="10"/>
       <c r="BP12" s="10"/>
       <c r="BR12" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS12" s="10"/>
-      <c r="BT12" s="10"/>
-      <c r="BU12" s="10"/>
-      <c r="BV12" s="10"/>
-      <c r="BW12" s="10"/>
-      <c r="BX12" s="10"/>
-      <c r="BY12" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY12" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA12" s="2" t="str">
         <f aca="false">IF(AS12="x","x",IF(AS12="-","-",""))</f>
         <v>x</v>
@@ -6703,15 +6712,29 @@
       <c r="BO13" s="10"/>
       <c r="BP13" s="10"/>
       <c r="BR13" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS13" s="10"/>
-      <c r="BT13" s="10"/>
-      <c r="BU13" s="10"/>
-      <c r="BV13" s="10"/>
-      <c r="BW13" s="10"/>
-      <c r="BX13" s="10"/>
-      <c r="BY13" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS13" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT13" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU13" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV13" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW13" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX13" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY13" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA13" s="2" t="str">
         <f aca="false">IF(AS13="x","x",IF(AS13="-","-",""))</f>
         <v>x</v>
@@ -7065,15 +7088,29 @@
       <c r="BO14" s="10"/>
       <c r="BP14" s="10"/>
       <c r="BR14" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS14" s="10"/>
-      <c r="BT14" s="10"/>
-      <c r="BU14" s="10"/>
-      <c r="BV14" s="10"/>
-      <c r="BW14" s="10"/>
-      <c r="BX14" s="10"/>
-      <c r="BY14" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX14" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY14" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA14" s="2" t="str">
         <f aca="false">IF(AS14="x","x",IF(AS14="-","-",""))</f>
         <v/>
@@ -7425,15 +7462,29 @@
       <c r="BO15" s="10"/>
       <c r="BP15" s="10"/>
       <c r="BR15" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS15" s="10"/>
-      <c r="BT15" s="10"/>
-      <c r="BU15" s="10"/>
-      <c r="BV15" s="10"/>
-      <c r="BW15" s="10"/>
-      <c r="BX15" s="10"/>
-      <c r="BY15" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY15" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA15" s="2" t="str">
         <f aca="false">IF(AS15="x","x",IF(AS15="-","-",""))</f>
         <v/>
@@ -7785,15 +7836,29 @@
       <c r="BO16" s="10"/>
       <c r="BP16" s="10"/>
       <c r="BR16" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS16" s="10"/>
-      <c r="BT16" s="10"/>
-      <c r="BU16" s="10"/>
-      <c r="BV16" s="10"/>
-      <c r="BW16" s="10"/>
-      <c r="BX16" s="10"/>
-      <c r="BY16" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX16" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY16" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA16" s="2" t="str">
         <f aca="false">IF(AS16="x","x",IF(AS16="-","-",""))</f>
         <v/>
@@ -8145,15 +8210,29 @@
       <c r="BO17" s="10"/>
       <c r="BP17" s="10"/>
       <c r="BR17" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS17" s="10"/>
-      <c r="BT17" s="10"/>
-      <c r="BU17" s="10"/>
-      <c r="BV17" s="10"/>
-      <c r="BW17" s="10"/>
-      <c r="BX17" s="10"/>
-      <c r="BY17" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY17" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA17" s="2" t="str">
         <f aca="false">IF(AS17="x","x",IF(AS17="-","-",""))</f>
         <v/>
@@ -8507,15 +8586,29 @@
       <c r="BO18" s="10"/>
       <c r="BP18" s="10"/>
       <c r="BR18" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS18" s="10"/>
-      <c r="BT18" s="10"/>
-      <c r="BU18" s="10"/>
-      <c r="BV18" s="10"/>
-      <c r="BW18" s="10"/>
-      <c r="BX18" s="10"/>
-      <c r="BY18" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX18" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY18" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA18" s="2" t="str">
         <f aca="false">IF(AS18="x","x",IF(AS18="-","-",""))</f>
         <v/>
@@ -8869,15 +8962,29 @@
       <c r="BO19" s="10"/>
       <c r="BP19" s="10"/>
       <c r="BR19" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS19" s="10"/>
-      <c r="BT19" s="10"/>
-      <c r="BU19" s="10"/>
-      <c r="BV19" s="10"/>
-      <c r="BW19" s="10"/>
-      <c r="BX19" s="10"/>
-      <c r="BY19" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY19" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA19" s="2" t="str">
         <f aca="false">IF(AS19="x","x",IF(AS19="-","-",""))</f>
         <v/>
@@ -9231,15 +9338,29 @@
       <c r="BO20" s="10"/>
       <c r="BP20" s="10"/>
       <c r="BR20" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS20" s="10"/>
-      <c r="BT20" s="10"/>
-      <c r="BU20" s="10"/>
-      <c r="BV20" s="10"/>
-      <c r="BW20" s="10"/>
-      <c r="BX20" s="10"/>
-      <c r="BY20" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX20" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY20" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA20" s="2" t="str">
         <f aca="false">IF(AS20="x","x",IF(AS20="-","-",""))</f>
         <v/>
@@ -9593,15 +9714,29 @@
       <c r="BO21" s="10"/>
       <c r="BP21" s="10"/>
       <c r="BR21" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS21" s="10"/>
-      <c r="BT21" s="10"/>
-      <c r="BU21" s="10"/>
-      <c r="BV21" s="10"/>
-      <c r="BW21" s="10"/>
-      <c r="BX21" s="10"/>
-      <c r="BY21" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX21" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY21" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA21" s="2" t="str">
         <f aca="false">IF(AS21="x","x",IF(AS21="-","-",""))</f>
         <v/>
@@ -9955,15 +10090,29 @@
       <c r="BO22" s="10"/>
       <c r="BP22" s="10"/>
       <c r="BR22" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS22" s="10"/>
-      <c r="BT22" s="10"/>
-      <c r="BU22" s="10"/>
-      <c r="BV22" s="10"/>
-      <c r="BW22" s="10"/>
-      <c r="BX22" s="10"/>
-      <c r="BY22" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX22" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY22" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA22" s="2" t="str">
         <f aca="false">IF(AS22="x","x",IF(AS22="-","-",""))</f>
         <v/>
@@ -10317,15 +10466,29 @@
       <c r="BO23" s="10"/>
       <c r="BP23" s="10"/>
       <c r="BR23" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS23" s="10"/>
-      <c r="BT23" s="10"/>
-      <c r="BU23" s="10"/>
-      <c r="BV23" s="10"/>
-      <c r="BW23" s="10"/>
-      <c r="BX23" s="10"/>
-      <c r="BY23" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX23" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY23" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA23" s="2" t="str">
         <f aca="false">IF(AS23="x","x",IF(AS23="-","-",""))</f>
         <v/>
@@ -10679,15 +10842,29 @@
       <c r="BO24" s="10"/>
       <c r="BP24" s="10"/>
       <c r="BR24" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS24" s="10"/>
-      <c r="BT24" s="10"/>
-      <c r="BU24" s="10"/>
-      <c r="BV24" s="10"/>
-      <c r="BW24" s="10"/>
-      <c r="BX24" s="10"/>
-      <c r="BY24" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX24" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY24" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA24" s="2" t="str">
         <f aca="false">IF(AS24="x","x",IF(AS24="-","-",""))</f>
         <v/>
@@ -11041,15 +11218,29 @@
       <c r="BO25" s="10"/>
       <c r="BP25" s="10"/>
       <c r="BR25" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS25" s="10"/>
-      <c r="BT25" s="10"/>
-      <c r="BU25" s="10"/>
-      <c r="BV25" s="10"/>
-      <c r="BW25" s="10"/>
-      <c r="BX25" s="10"/>
-      <c r="BY25" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS25" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT25" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU25" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV25" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW25" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX25" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY25" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA25" s="2" t="str">
         <f aca="false">IF(AS25="x","x",IF(AS25="-","-",""))</f>
         <v/>
@@ -11403,15 +11594,29 @@
       <c r="BO26" s="10"/>
       <c r="BP26" s="10"/>
       <c r="BR26" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS26" s="10"/>
-      <c r="BT26" s="10"/>
-      <c r="BU26" s="10"/>
-      <c r="BV26" s="10"/>
-      <c r="BW26" s="10"/>
-      <c r="BX26" s="10"/>
-      <c r="BY26" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX26" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY26" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA26" s="2" t="str">
         <f aca="false">IF(AS26="x","x",IF(AS26="-","-",""))</f>
         <v/>
@@ -11765,15 +11970,29 @@
       <c r="BO27" s="10"/>
       <c r="BP27" s="10"/>
       <c r="BR27" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS27" s="10"/>
-      <c r="BT27" s="10"/>
-      <c r="BU27" s="10"/>
-      <c r="BV27" s="10"/>
-      <c r="BW27" s="10"/>
-      <c r="BX27" s="10"/>
-      <c r="BY27" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX27" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY27" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA27" s="2" t="str">
         <f aca="false">IF(AS27="x","x",IF(AS27="-","-",""))</f>
         <v/>
@@ -12121,15 +12340,29 @@
       <c r="BO28" s="10"/>
       <c r="BP28" s="10"/>
       <c r="BR28" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS28" s="10"/>
-      <c r="BT28" s="10"/>
-      <c r="BU28" s="10"/>
-      <c r="BV28" s="10"/>
-      <c r="BW28" s="10"/>
-      <c r="BX28" s="10"/>
-      <c r="BY28" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY28" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA28" s="2" t="str">
         <f aca="false">IF(AS28="x","x",IF(AS28="-","-",""))</f>
         <v/>
@@ -12483,15 +12716,29 @@
       <c r="BO29" s="10"/>
       <c r="BP29" s="10"/>
       <c r="BR29" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS29" s="10"/>
-      <c r="BT29" s="10"/>
-      <c r="BU29" s="10"/>
-      <c r="BV29" s="10"/>
-      <c r="BW29" s="10"/>
-      <c r="BX29" s="10"/>
-      <c r="BY29" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY29" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA29" s="2" t="str">
         <f aca="false">IF(AS29="x","x",IF(AS29="-","-",""))</f>
         <v/>
@@ -12845,15 +13092,29 @@
       <c r="BO30" s="10"/>
       <c r="BP30" s="10"/>
       <c r="BR30" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS30" s="10"/>
-      <c r="BT30" s="10"/>
-      <c r="BU30" s="10"/>
-      <c r="BV30" s="10"/>
-      <c r="BW30" s="10"/>
-      <c r="BX30" s="10"/>
-      <c r="BY30" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS30" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT30" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU30" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV30" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW30" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX30" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY30" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA30" s="2" t="str">
         <f aca="false">IF(AS30="x","x",IF(AS30="-","-",""))</f>
         <v/>
@@ -13207,15 +13468,29 @@
       <c r="BO31" s="10"/>
       <c r="BP31" s="10"/>
       <c r="BR31" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS31" s="10"/>
-      <c r="BT31" s="10"/>
-      <c r="BU31" s="10"/>
-      <c r="BV31" s="10"/>
-      <c r="BW31" s="10"/>
-      <c r="BX31" s="10"/>
-      <c r="BY31" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS31" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT31" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU31" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV31" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW31" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX31" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY31" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA31" s="2" t="str">
         <f aca="false">IF(AS31="x","x",IF(AS31="-","-",""))</f>
         <v/>
@@ -13569,15 +13844,29 @@
       <c r="BO32" s="10"/>
       <c r="BP32" s="10"/>
       <c r="BR32" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS32" s="10"/>
-      <c r="BT32" s="10"/>
-      <c r="BU32" s="10"/>
-      <c r="BV32" s="10"/>
-      <c r="BW32" s="10"/>
-      <c r="BX32" s="10"/>
-      <c r="BY32" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS32" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT32" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU32" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV32" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW32" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX32" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY32" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA32" s="2" t="str">
         <f aca="false">IF(AS32="x","x",IF(AS32="-","-",""))</f>
         <v/>
@@ -13931,15 +14220,29 @@
       <c r="BO33" s="10"/>
       <c r="BP33" s="10"/>
       <c r="BR33" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS33" s="10"/>
-      <c r="BT33" s="10"/>
-      <c r="BU33" s="10"/>
-      <c r="BV33" s="10"/>
-      <c r="BW33" s="10"/>
-      <c r="BX33" s="10"/>
-      <c r="BY33" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS33" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT33" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU33" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV33" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW33" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX33" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY33" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA33" s="2" t="str">
         <f aca="false">IF(AS33="x","x",IF(AS33="-","-",""))</f>
         <v/>
@@ -14293,15 +14596,29 @@
       <c r="BO34" s="10"/>
       <c r="BP34" s="10"/>
       <c r="BR34" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS34" s="10"/>
-      <c r="BT34" s="10"/>
-      <c r="BU34" s="10"/>
-      <c r="BV34" s="10"/>
-      <c r="BW34" s="10"/>
-      <c r="BX34" s="10"/>
-      <c r="BY34" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS34" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT34" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU34" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV34" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW34" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX34" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY34" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA34" s="2" t="str">
         <f aca="false">IF(AS34="x","x",IF(AS34="-","-",""))</f>
         <v/>
@@ -14655,15 +14972,29 @@
       <c r="BO35" s="10"/>
       <c r="BP35" s="10"/>
       <c r="BR35" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS35" s="10"/>
-      <c r="BT35" s="10"/>
-      <c r="BU35" s="10"/>
-      <c r="BV35" s="10"/>
-      <c r="BW35" s="10"/>
-      <c r="BX35" s="10"/>
-      <c r="BY35" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX35" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY35" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA35" s="2" t="str">
         <f aca="false">IF(AS35="x","x",IF(AS35="-","-",""))</f>
         <v/>
@@ -15017,15 +15348,29 @@
       <c r="BO36" s="10"/>
       <c r="BP36" s="10"/>
       <c r="BR36" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS36" s="10"/>
-      <c r="BT36" s="10"/>
-      <c r="BU36" s="10"/>
-      <c r="BV36" s="10"/>
-      <c r="BW36" s="10"/>
-      <c r="BX36" s="10"/>
-      <c r="BY36" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY36" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA36" s="2" t="str">
         <f aca="false">IF(AS36="x","x",IF(AS36="-","-",""))</f>
         <v/>
@@ -15379,15 +15724,29 @@
       <c r="BO37" s="10"/>
       <c r="BP37" s="10"/>
       <c r="BR37" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS37" s="10"/>
-      <c r="BT37" s="10"/>
-      <c r="BU37" s="10"/>
-      <c r="BV37" s="10"/>
-      <c r="BW37" s="10"/>
-      <c r="BX37" s="10"/>
-      <c r="BY37" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX37" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY37" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA37" s="2" t="str">
         <f aca="false">IF(AS37="x","x",IF(AS37="-","-",""))</f>
         <v/>
@@ -15739,15 +16098,29 @@
       <c r="BO38" s="10"/>
       <c r="BP38" s="10"/>
       <c r="BR38" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS38" s="10"/>
-      <c r="BT38" s="10"/>
-      <c r="BU38" s="10"/>
-      <c r="BV38" s="10"/>
-      <c r="BW38" s="10"/>
-      <c r="BX38" s="10"/>
-      <c r="BY38" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS38" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT38" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU38" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV38" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW38" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX38" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY38" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA38" s="2" t="str">
         <f aca="false">IF(AS38="x","x",IF(AS38="-","-",""))</f>
         <v/>
@@ -16099,15 +16472,29 @@
       <c r="BO39" s="10"/>
       <c r="BP39" s="10"/>
       <c r="BR39" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS39" s="10"/>
-      <c r="BT39" s="10"/>
-      <c r="BU39" s="10"/>
-      <c r="BV39" s="10"/>
-      <c r="BW39" s="10"/>
-      <c r="BX39" s="10"/>
-      <c r="BY39" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS39" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT39" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU39" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV39" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW39" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX39" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY39" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA39" s="2" t="str">
         <f aca="false">IF(AS39="x","x",IF(AS39="-","-",""))</f>
         <v/>
@@ -16459,15 +16846,29 @@
       <c r="BO40" s="10"/>
       <c r="BP40" s="10"/>
       <c r="BR40" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS40" s="10"/>
-      <c r="BT40" s="10"/>
-      <c r="BU40" s="10"/>
-      <c r="BV40" s="10"/>
-      <c r="BW40" s="10"/>
-      <c r="BX40" s="10"/>
-      <c r="BY40" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS40" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT40" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU40" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV40" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW40" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX40" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY40" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA40" s="2" t="str">
         <f aca="false">IF(AS40="x","x",IF(AS40="-","-",""))</f>
         <v/>
@@ -16819,15 +17220,29 @@
       <c r="BO41" s="10"/>
       <c r="BP41" s="10"/>
       <c r="BR41" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BS41" s="10"/>
-      <c r="BT41" s="10"/>
-      <c r="BU41" s="10"/>
-      <c r="BV41" s="10"/>
-      <c r="BW41" s="10"/>
-      <c r="BX41" s="10"/>
-      <c r="BY41" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BS41" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BT41" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU41" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV41" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW41" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX41" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY41" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA41" s="2" t="str">
         <f aca="false">IF(AS41="x","x",IF(AS41="-","-",""))</f>
         <v/>
@@ -17180,16 +17595,30 @@
       <c r="BN42" s="10"/>
       <c r="BO42" s="10"/>
       <c r="BP42" s="10"/>
-      <c r="BR42" s="10"/>
+      <c r="BR42" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS42" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT42" s="10"/>
-      <c r="BU42" s="10"/>
-      <c r="BV42" s="10"/>
-      <c r="BW42" s="10"/>
-      <c r="BX42" s="10"/>
-      <c r="BY42" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT42" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU42" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV42" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW42" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX42" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY42" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA42" s="2" t="str">
         <f aca="false">IF(AS42="x","x",IF(AS42="-","-",""))</f>
         <v/>
@@ -17542,16 +17971,30 @@
       <c r="BN43" s="10"/>
       <c r="BO43" s="10"/>
       <c r="BP43" s="10"/>
-      <c r="BR43" s="10"/>
+      <c r="BR43" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS43" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT43" s="10"/>
-      <c r="BU43" s="10"/>
-      <c r="BV43" s="10"/>
-      <c r="BW43" s="10"/>
-      <c r="BX43" s="10"/>
-      <c r="BY43" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT43" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU43" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV43" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW43" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX43" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY43" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA43" s="2" t="str">
         <f aca="false">IF(AS43="x","x",IF(AS43="-","-",""))</f>
         <v/>
@@ -17904,16 +18347,30 @@
       <c r="BN44" s="10"/>
       <c r="BO44" s="10"/>
       <c r="BP44" s="10"/>
-      <c r="BR44" s="10"/>
+      <c r="BR44" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS44" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT44" s="10"/>
-      <c r="BU44" s="10"/>
-      <c r="BV44" s="10"/>
-      <c r="BW44" s="10"/>
-      <c r="BX44" s="10"/>
-      <c r="BY44" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT44" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU44" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV44" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW44" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX44" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY44" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA44" s="2" t="str">
         <f aca="false">IF(AS44="x","x",IF(AS44="-","-",""))</f>
         <v/>
@@ -18266,16 +18723,30 @@
       <c r="BN45" s="10"/>
       <c r="BO45" s="10"/>
       <c r="BP45" s="10"/>
-      <c r="BR45" s="10"/>
+      <c r="BR45" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS45" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT45" s="10"/>
-      <c r="BU45" s="10"/>
-      <c r="BV45" s="10"/>
-      <c r="BW45" s="10"/>
-      <c r="BX45" s="10"/>
-      <c r="BY45" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT45" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU45" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV45" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW45" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX45" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY45" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA45" s="2" t="str">
         <f aca="false">IF(AS45="x","x",IF(AS45="-","-",""))</f>
         <v/>
@@ -18628,16 +19099,30 @@
       <c r="BN46" s="10"/>
       <c r="BO46" s="10"/>
       <c r="BP46" s="10"/>
-      <c r="BR46" s="10"/>
+      <c r="BR46" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS46" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT46" s="10"/>
-      <c r="BU46" s="10"/>
-      <c r="BV46" s="10"/>
-      <c r="BW46" s="10"/>
-      <c r="BX46" s="10"/>
-      <c r="BY46" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT46" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU46" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV46" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW46" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX46" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY46" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA46" s="2" t="str">
         <f aca="false">IF(AS46="x","x",IF(AS46="-","-",""))</f>
         <v/>
@@ -18990,16 +19475,30 @@
       <c r="BN47" s="10"/>
       <c r="BO47" s="10"/>
       <c r="BP47" s="10"/>
-      <c r="BR47" s="10"/>
+      <c r="BR47" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS47" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT47" s="10"/>
-      <c r="BU47" s="10"/>
-      <c r="BV47" s="10"/>
-      <c r="BW47" s="10"/>
-      <c r="BX47" s="10"/>
-      <c r="BY47" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT47" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU47" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV47" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW47" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX47" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY47" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA47" s="2" t="str">
         <f aca="false">IF(AS47="x","x",IF(AS47="-","-",""))</f>
         <v/>
@@ -19352,16 +19851,30 @@
       <c r="BN48" s="10"/>
       <c r="BO48" s="10"/>
       <c r="BP48" s="10"/>
-      <c r="BR48" s="10"/>
+      <c r="BR48" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS48" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT48" s="10"/>
-      <c r="BU48" s="10"/>
-      <c r="BV48" s="10"/>
-      <c r="BW48" s="10"/>
-      <c r="BX48" s="10"/>
-      <c r="BY48" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT48" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU48" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV48" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW48" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX48" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY48" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA48" s="2" t="str">
         <f aca="false">IF(AS48="x","x",IF(AS48="-","-",""))</f>
         <v/>
@@ -19714,16 +20227,30 @@
       <c r="BN49" s="10"/>
       <c r="BO49" s="10"/>
       <c r="BP49" s="10"/>
-      <c r="BR49" s="10"/>
+      <c r="BR49" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="BS49" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="BT49" s="10"/>
-      <c r="BU49" s="10"/>
-      <c r="BV49" s="10"/>
-      <c r="BW49" s="10"/>
-      <c r="BX49" s="10"/>
-      <c r="BY49" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="BT49" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BU49" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV49" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BW49" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BX49" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="BY49" s="10" t="s">
+        <v>77</v>
+      </c>
       <c r="CA49" s="2" t="str">
         <f aca="false">IF(AS49="x","x",IF(AS49="-","-",""))</f>
         <v/>

</xml_diff>